<commit_message>
V5: coupled dielectric + catheter heating GUI
- V5_convection/Coupled_heating_GUI: v5_gui (two tabs, modal exact-in-time
  solver, power envelope, registered photographs) with v5_selftest
- v5_gui adds its own folder to the path and keeps the figure handle, so it
  works from VS Code's Run button (cwd = repo root)
- power envelope axes can be panned/zoomed; zoom survives setting changes
- supporting derivations, E-field script, convection model docx, setup table
- ignore GUI exports and Office lock files

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Gel_model_V3/Experimental_setup_table.xlsx
+++ b/Gel_model_V3/Experimental_setup_table.xlsx
@@ -614,6 +614,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="afd333ce-61b4-499e-a6b0-4856631dff3b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F6C796F03D00A6439A212FBC48167B84" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="51cbcf33217eb0a68bf1d80dce202c35">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="afd333ce-61b4-499e-a6b0-4856631dff3b" xmlns:ns4="91d970ef-24a4-4d9d-98d3-63f44481be54" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e28ca76a09000554ff21e86f69c5f96e" ns3:_="" ns4:_="">
     <xsd:import namespace="afd333ce-61b4-499e-a6b0-4856631dff3b"/>
@@ -834,7 +842,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -843,15 +851,24 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="afd333ce-61b4-499e-a6b0-4856631dff3b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08F6B934-84EF-495D-B5DF-644B32E5B3B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="91d970ef-24a4-4d9d-98d3-63f44481be54"/>
+    <ds:schemaRef ds:uri="afd333ce-61b4-499e-a6b0-4856631dff3b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21480140-773E-4C23-BFC0-BB9C9E2BA2CA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -870,27 +887,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{046C4BCF-1CB7-4EBF-8006-16FD0A03B688}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08F6B934-84EF-495D-B5DF-644B32E5B3B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="91d970ef-24a4-4d9d-98d3-63f44481be54"/>
-    <ds:schemaRef ds:uri="afd333ce-61b4-499e-a6b0-4856631dff3b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>